<commit_message>
Account tab titles: add holdings date
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_23.10.2026.xlsx
+++ b/Consolidated_Portfolios_23.10.2026.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="283">
   <si>
     <t xml:space="preserve">CONSOLIDATED PORTFOLIO SUMMARY – ALL MANAGED ACCOUNTS</t>
   </si>
@@ -633,6 +633,9 @@
     <t xml:space="preserve">No exchange close found – statement price used</t>
   </si>
   <si>
+    <t xml:space="preserve">GAUTAM – HDFC Securities – 23.10.2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">Holdings as of 23.10.2026. Statement prices: HDFC statement prices 23.10.2026. Market value uses the common Ref Price from the Prices sheet so all portfolios are valued alike.</t>
   </si>
   <si>
@@ -706,6 +709,9 @@
   </si>
   <si>
     <t xml:space="preserve">No cost or price on statement (marked *) – carried at nil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANISH SHILPA – Axis Direct + HDFC Securities – 23.10.2026 (live, ~11:23 IST)</t>
   </si>
   <si>
     <t xml:space="preserve">Holdings as of 23.10.2026 (live, ~11:23 IST). Statement prices: Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged). Market value uses the common Ref Price from the Prices sheet so all portfolios are valued alike.</t>
@@ -795,6 +801,9 @@
     <t xml:space="preserve">Axis Direct Shilpa 1; Axis Direct Manish 4</t>
   </si>
   <si>
+    <t xml:space="preserve">SALONI MEHRA – Angel One – 20.10.2026 + trades of 21–23.10.2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">Holdings as of 20.10.2026 + trades of 21–23.10.2026. Statement prices: 20.10.2026 statement prices (only for rows with no trades since). Market value uses the common Ref Price from the Prices sheet so all portfolios are valued alike.</t>
   </si>
   <si>
@@ -846,6 +855,9 @@
     <t xml:space="preserve">New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known</t>
   </si>
   <si>
+    <t xml:space="preserve">VIDUSHI MALHOTRA – Zerodha – 04.10.2026 (+ trades of 05.10.2026)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Holdings as of 04.10.2026 (+ trades of 05.10.2026). Statement prices: LTP 05.10.2026. Market value uses the common Ref Price from the Prices sheet so all portfolios are valued alike.</t>
   </si>
   <si>
@@ -859,6 +871,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-05 12:46:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DR UMESH CHOUDHRY – ICICI Direct – 04.10.2026 + trades of 09.10.2026</t>
   </si>
   <si>
     <t xml:space="preserve">Holdings as of 04.10.2026 + trades of 09.10.2026. Statement prices: NSE live 09.10.2026 ~09:45 IST. Market value uses the common Ref Price from the Prices sheet so all portfolios are valued alike.</t>
@@ -877,6 +892,9 @@
   </si>
   <si>
     <t xml:space="preserve">New position 09.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DA – HDFC Securities + Kotak Securities – Post 12.09.2026 trades (file dated 04.10.2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Holdings as of Post 12.09.2026 trades (file dated 04.10.2026). Statement prices: As on statement (date not printed). Market value uses the common Ref Price from the Prices sheet so all portfolios are valued alike.</t>
@@ -2935,12 +2953,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -27225,22 +27243,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="32" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27248,16 +27266,16 @@
         <v>69</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C6" s="23" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F6" s="23" t="s">
         <v>74</v>
@@ -27275,37 +27293,37 @@
         <v>10</v>
       </c>
       <c r="K6" s="23" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L6" s="23" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="M6" s="23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N6" s="23" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O6" s="23" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="Q6" s="23" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="R6" s="23" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="S6" s="23" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="T6" s="23" t="s">
         <v>73</v>
       </c>
       <c r="U6" s="23" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="V6" s="23" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27361,10 +27379,10 @@
       </c>
       <c r="O7" s="67"/>
       <c r="Q7" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R7" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S7" s="68" t="s">
         <v>94</v>
@@ -27432,10 +27450,10 @@
       </c>
       <c r="O8" s="67"/>
       <c r="Q8" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R8" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S8" s="68" t="s">
         <v>102</v>
@@ -27503,10 +27521,10 @@
       </c>
       <c r="O9" s="67"/>
       <c r="Q9" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R9" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S9" s="68" t="s">
         <v>79</v>
@@ -27574,10 +27592,10 @@
       </c>
       <c r="O10" s="67"/>
       <c r="Q10" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R10" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S10" s="68" t="s">
         <v>86</v>
@@ -27644,13 +27662,13 @@
         <v>0</v>
       </c>
       <c r="O11" s="67" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q11" s="68" t="s">
+        <v>202</v>
+      </c>
+      <c r="R11" s="68" t="s">
         <v>203</v>
-      </c>
-      <c r="Q11" s="68" t="s">
-        <v>201</v>
-      </c>
-      <c r="R11" s="68" t="s">
-        <v>202</v>
       </c>
       <c r="S11" s="68" t="s">
         <v>96</v>
@@ -27718,10 +27736,10 @@
       </c>
       <c r="O12" s="67"/>
       <c r="Q12" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R12" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S12" s="68" t="s">
         <v>91</v>
@@ -27789,10 +27807,10 @@
       </c>
       <c r="O13" s="67"/>
       <c r="Q13" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R13" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S13" s="68" t="s">
         <v>83</v>
@@ -27860,13 +27878,13 @@
       </c>
       <c r="O14" s="67"/>
       <c r="Q14" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R14" s="68" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="S14" s="68" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="T14" s="68" t="n">
         <v>80</v>
@@ -27930,13 +27948,13 @@
         <v>-666</v>
       </c>
       <c r="O15" s="67" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Q15" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R15" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S15" s="68" t="s">
         <v>88</v>
@@ -28004,10 +28022,10 @@
       </c>
       <c r="O16" s="67"/>
       <c r="Q16" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R16" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S16" s="68" t="s">
         <v>95</v>
@@ -28075,10 +28093,10 @@
       </c>
       <c r="O17" s="67"/>
       <c r="Q17" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R17" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S17" s="68" t="s">
         <v>93</v>
@@ -28146,10 +28164,10 @@
       </c>
       <c r="O18" s="67"/>
       <c r="Q18" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R18" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S18" s="68" t="s">
         <v>82</v>
@@ -28217,10 +28235,10 @@
       </c>
       <c r="O19" s="67"/>
       <c r="Q19" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R19" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S19" s="68" t="s">
         <v>104</v>
@@ -28288,10 +28306,10 @@
       </c>
       <c r="O20" s="67"/>
       <c r="Q20" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R20" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S20" s="68" t="s">
         <v>92</v>
@@ -28358,13 +28376,13 @@
         <v>-160</v>
       </c>
       <c r="O21" s="67" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q21" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R21" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S21" s="68" t="s">
         <v>80</v>
@@ -28432,10 +28450,10 @@
       </c>
       <c r="O22" s="67"/>
       <c r="Q22" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R22" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S22" s="68" t="s">
         <v>100</v>
@@ -28503,10 +28521,10 @@
       </c>
       <c r="O23" s="67"/>
       <c r="Q23" s="68" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R23" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S23" s="68" t="s">
         <v>105</v>
@@ -28574,7 +28592,7 @@
       </c>
       <c r="O24" s="67"/>
       <c r="S24" s="69" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="V24" s="70" t="n">
         <f aca="false">SUMIFS(V7:V23,R7:R23,"BUY")-SUMIFS(V7:V23,R7:R23,"SELL")</f>
@@ -29212,7 +29230,7 @@
         <v/>
       </c>
       <c r="O36" s="78" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29263,7 +29281,7 @@
         <v/>
       </c>
       <c r="O37" s="78" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29341,17 +29359,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29359,16 +29377,16 @@
         <v>69</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F6" s="24" t="s">
         <v>74</v>
@@ -29386,19 +29404,19 @@
         <v>10</v>
       </c>
       <c r="K6" s="24" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L6" s="24" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="M6" s="24" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N6" s="24" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O6" s="24" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29409,7 +29427,7 @@
         <v>79</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D7" s="66" t="n">
         <v>3895</v>
@@ -29453,7 +29471,7 @@
         <v>43579.5</v>
       </c>
       <c r="O7" s="67" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29464,7 +29482,7 @@
         <v>81</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D8" s="66" t="n">
         <v>11160</v>
@@ -29508,7 +29526,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="67" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29519,7 +29537,7 @@
         <v>80</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D9" s="66" t="n">
         <v>165</v>
@@ -29563,7 +29581,7 @@
         <v>17025</v>
       </c>
       <c r="O9" s="67" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29574,7 +29592,7 @@
         <v>83</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D10" s="66" t="n">
         <v>1013</v>
@@ -29618,7 +29636,7 @@
         <v>5129.64999999991</v>
       </c>
       <c r="O10" s="67" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29629,7 +29647,7 @@
         <v>82</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D11" s="66" t="n">
         <v>1394</v>
@@ -29673,7 +29691,7 @@
         <v>24777.2999999999</v>
       </c>
       <c r="O11" s="67" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29684,7 +29702,7 @@
         <v>84</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D12" s="66" t="n">
         <v>360</v>
@@ -29737,7 +29755,7 @@
         <v>97</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D13" s="66" t="n">
         <v>2004.589</v>
@@ -29781,7 +29799,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="67" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29792,7 +29810,7 @@
         <v>86</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D14" s="66" t="n">
         <v>3762</v>
@@ -29836,7 +29854,7 @@
         <v>12713.24</v>
       </c>
       <c r="O14" s="67" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29847,7 +29865,7 @@
         <v>88</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D15" s="66" t="n">
         <v>72</v>
@@ -29891,7 +29909,7 @@
         <v>2157.60000000004</v>
       </c>
       <c r="O15" s="67" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29902,7 +29920,7 @@
         <v>87</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D16" s="66" t="n">
         <v>66</v>
@@ -29946,7 +29964,7 @@
         <v>5268</v>
       </c>
       <c r="O16" s="67" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29957,7 +29975,7 @@
         <v>89</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D17" s="66" t="n">
         <v>800</v>
@@ -30010,7 +30028,7 @@
         <v>91</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D18" s="66" t="n">
         <v>3500</v>
@@ -30063,7 +30081,7 @@
         <v>103</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D19" s="66" t="n">
         <v>134</v>
@@ -30116,7 +30134,7 @@
         <v>92</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D20" s="66" t="n">
         <v>32</v>
@@ -30160,7 +30178,7 @@
         <v>2627.60000000001</v>
       </c>
       <c r="O20" s="67" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30171,7 +30189,7 @@
         <v>109</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D21" s="66" t="n">
         <v>44</v>
@@ -30224,7 +30242,7 @@
         <v>110</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D22" s="66" t="n">
         <v>3</v>
@@ -30277,7 +30295,7 @@
         <v>111</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D23" s="66" t="n">
         <v>64</v>
@@ -30330,7 +30348,7 @@
         <v>85</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D24" s="66" t="n">
         <v>29</v>
@@ -30383,7 +30401,7 @@
         <v>112</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D25" s="66" t="n">
         <v>160</v>
@@ -30427,7 +30445,7 @@
         <v>622</v>
       </c>
       <c r="O25" s="67" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30438,7 +30456,7 @@
         <v>113</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D26" s="66" t="n">
         <v>2</v>
@@ -30491,7 +30509,7 @@
         <v>94</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D27" s="66" t="n">
         <v>47</v>
@@ -30535,7 +30553,7 @@
         <v>1797.6</v>
       </c>
       <c r="O27" s="67" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30546,7 +30564,7 @@
         <v>93</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D28" s="66" t="n">
         <v>11</v>
@@ -30590,7 +30608,7 @@
         <v>-502.5</v>
       </c>
       <c r="O28" s="67" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30601,7 +30619,7 @@
         <v>115</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D29" s="66" t="n">
         <v>22</v>
@@ -30654,7 +30672,7 @@
         <v>96</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D30" s="66" t="n">
         <v>6</v>
@@ -30698,7 +30716,7 @@
         <v>747</v>
       </c>
       <c r="O30" s="67" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30709,7 +30727,7 @@
         <v>99</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D31" s="66" t="n">
         <v>32</v>
@@ -30762,7 +30780,7 @@
         <v>125</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D32" s="66" t="n">
         <v>34</v>
@@ -30815,7 +30833,7 @@
         <v>100</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D33" s="66" t="n">
         <v>10</v>
@@ -30859,7 +30877,7 @@
         <v>628</v>
       </c>
       <c r="O33" s="67" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30870,7 +30888,7 @@
         <v>118</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D34" s="66" t="n">
         <v>168</v>
@@ -30914,7 +30932,7 @@
         <v>1205</v>
       </c>
       <c r="O34" s="67" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30925,7 +30943,7 @@
         <v>135</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D35" s="66" t="n">
         <v>33</v>
@@ -30978,7 +30996,7 @@
         <v>102</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D36" s="66" t="n">
         <v>6</v>
@@ -31022,7 +31040,7 @@
         <v>238</v>
       </c>
       <c r="O36" s="67" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31033,7 +31051,7 @@
         <v>101</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D37" s="66" t="n">
         <v>17</v>
@@ -31077,7 +31095,7 @@
         <v>386.300000000003</v>
       </c>
       <c r="O37" s="67" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31088,7 +31106,7 @@
         <v>105</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D38" s="66" t="n">
         <v>6</v>
@@ -31132,7 +31150,7 @@
         <v>320</v>
       </c>
       <c r="O38" s="67" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31143,7 +31161,7 @@
         <v>148</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D39" s="66" t="n">
         <v>50</v>
@@ -31196,7 +31214,7 @@
         <v>150</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D40" s="66" t="n">
         <v>35</v>
@@ -31249,7 +31267,7 @@
         <v>151</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D41" s="66" t="n">
         <v>14</v>
@@ -31302,7 +31320,7 @@
         <v>152</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D42" s="66" t="n">
         <v>34</v>
@@ -31346,7 +31364,7 @@
         <v>-59.7000000000007</v>
       </c>
       <c r="O42" s="67" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31357,7 +31375,7 @@
         <v>108</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D43" s="66" t="n">
         <v>32</v>
@@ -31410,7 +31428,7 @@
         <v>157</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D44" s="66" t="n">
         <v>3</v>
@@ -31463,7 +31481,7 @@
         <v>95</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D45" s="66" t="n">
         <v>4</v>
@@ -31507,7 +31525,7 @@
         <v>-1559</v>
       </c>
       <c r="O45" s="67" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31518,7 +31536,7 @@
         <v>104</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D46" s="66" t="n">
         <v>5</v>
@@ -31571,7 +31589,7 @@
         <v>159</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D47" s="66" t="n">
         <v>5</v>
@@ -31624,7 +31642,7 @@
         <v>160</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D48" s="66" t="n">
         <v>1</v>
@@ -31677,7 +31695,7 @@
         <v>155</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D49" s="66" t="n">
         <v>5</v>
@@ -31721,7 +31739,7 @@
         <v>196.75</v>
       </c>
       <c r="O49" s="67" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31732,7 +31750,7 @@
         <v>162</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D50" s="66" t="n">
         <v>6</v>
@@ -31785,7 +31803,7 @@
         <v>163</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D51" s="66" t="n">
         <v>1</v>
@@ -31838,7 +31856,7 @@
         <v>139</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D52" s="66" t="n">
         <v>12</v>
@@ -31891,7 +31909,7 @@
         <v>165</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D53" s="66" t="n">
         <v>5</v>
@@ -32017,22 +32035,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="32" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32040,16 +32058,16 @@
         <v>69</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C6" s="25" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F6" s="25" t="s">
         <v>74</v>
@@ -32067,37 +32085,37 @@
         <v>10</v>
       </c>
       <c r="K6" s="25" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L6" s="25" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N6" s="25" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O6" s="25" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="Q6" s="25" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="R6" s="25" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="S6" s="25" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="T6" s="25" t="s">
         <v>73</v>
       </c>
       <c r="U6" s="25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="V6" s="25" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32150,13 +32168,13 @@
         <v/>
       </c>
       <c r="O7" s="67" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="Q7" s="68" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="R7" s="68" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="S7" s="68" t="s">
         <v>112</v>
@@ -32221,13 +32239,13 @@
         <v/>
       </c>
       <c r="O8" s="67" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="Q8" s="68" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="R8" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S8" s="68" t="s">
         <v>86</v>
@@ -32292,13 +32310,13 @@
         <v/>
       </c>
       <c r="O9" s="67" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="Q9" s="68" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="R9" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S9" s="68" t="s">
         <v>80</v>
@@ -32366,10 +32384,10 @@
       </c>
       <c r="O10" s="67"/>
       <c r="Q10" s="68" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="R10" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S10" s="68" t="s">
         <v>83</v>
@@ -32434,13 +32452,13 @@
         <v/>
       </c>
       <c r="O11" s="67" t="s">
+        <v>248</v>
+      </c>
+      <c r="Q11" s="68" t="s">
         <v>245</v>
       </c>
-      <c r="Q11" s="68" t="s">
-        <v>242</v>
-      </c>
       <c r="R11" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S11" s="68" t="s">
         <v>82</v>
@@ -32508,13 +32526,13 @@
       </c>
       <c r="O12" s="67"/>
       <c r="Q12" s="68" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="R12" s="68" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="S12" s="68" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="T12" s="68" t="n">
         <v>700</v>
@@ -32579,10 +32597,10 @@
       </c>
       <c r="O13" s="67"/>
       <c r="Q13" s="68" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="R13" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S13" s="68" t="s">
         <v>79</v>
@@ -32650,10 +32668,10 @@
       </c>
       <c r="O14" s="67"/>
       <c r="Q14" s="68" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="R14" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S14" s="68" t="s">
         <v>93</v>
@@ -32718,13 +32736,13 @@
         <v/>
       </c>
       <c r="O15" s="67" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="Q15" s="68" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="R15" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S15" s="68" t="s">
         <v>92</v>
@@ -32789,13 +32807,13 @@
         <v/>
       </c>
       <c r="O16" s="67" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="Q16" s="68" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="R16" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S16" s="68" t="s">
         <v>88</v>
@@ -32863,10 +32881,10 @@
       </c>
       <c r="O17" s="67"/>
       <c r="Q17" s="68" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="R17" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S17" s="68" t="s">
         <v>100</v>
@@ -32931,13 +32949,13 @@
         <v/>
       </c>
       <c r="O18" s="67" t="s">
+        <v>253</v>
+      </c>
+      <c r="Q18" s="68" t="s">
         <v>250</v>
       </c>
-      <c r="Q18" s="68" t="s">
-        <v>247</v>
-      </c>
       <c r="R18" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S18" s="68" t="s">
         <v>94</v>
@@ -33002,13 +33020,13 @@
         <v/>
       </c>
       <c r="O19" s="67" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="Q19" s="68" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="R19" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S19" s="68" t="s">
         <v>96</v>
@@ -33076,10 +33094,10 @@
       </c>
       <c r="O20" s="67"/>
       <c r="Q20" s="68" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="R20" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S20" s="68" t="s">
         <v>102</v>
@@ -33144,13 +33162,13 @@
         <v/>
       </c>
       <c r="O21" s="67" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="Q21" s="68" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="R21" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S21" s="68" t="s">
         <v>104</v>
@@ -33215,13 +33233,13 @@
         <v/>
       </c>
       <c r="O22" s="67" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="Q22" s="68" t="s">
         <v>17</v>
       </c>
       <c r="R22" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S22" s="68" t="s">
         <v>91</v>
@@ -33286,13 +33304,13 @@
         <v/>
       </c>
       <c r="O23" s="67" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="Q23" s="68" t="s">
         <v>17</v>
       </c>
       <c r="R23" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S23" s="68" t="s">
         <v>101</v>
@@ -33357,13 +33375,13 @@
         <v/>
       </c>
       <c r="O24" s="67" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="Q24" s="68" t="s">
         <v>17</v>
       </c>
       <c r="R24" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S24" s="68" t="s">
         <v>155</v>
@@ -33428,13 +33446,13 @@
         <v/>
       </c>
       <c r="O25" s="67" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="Q25" s="68" t="s">
         <v>17</v>
       </c>
       <c r="R25" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S25" s="68" t="s">
         <v>105</v>
@@ -33499,13 +33517,13 @@
         <v/>
       </c>
       <c r="O26" s="67" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="Q26" s="68" t="s">
         <v>17</v>
       </c>
       <c r="R26" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S26" s="68" t="s">
         <v>106</v>
@@ -33570,13 +33588,13 @@
         <v/>
       </c>
       <c r="O27" s="67" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="Q27" s="68" t="s">
         <v>17</v>
       </c>
       <c r="R27" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S27" s="68" t="s">
         <v>102</v>
@@ -33641,13 +33659,13 @@
         <v/>
       </c>
       <c r="O28" s="67" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="Q28" s="68" t="s">
         <v>17</v>
       </c>
       <c r="R28" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S28" s="68" t="s">
         <v>100</v>
@@ -33712,13 +33730,13 @@
         <v/>
       </c>
       <c r="O29" s="67" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="Q29" s="68" t="s">
         <v>17</v>
       </c>
       <c r="R29" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S29" s="68" t="s">
         <v>96</v>
@@ -33783,13 +33801,13 @@
         <v/>
       </c>
       <c r="O30" s="67" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="Q30" s="68" t="s">
         <v>17</v>
       </c>
       <c r="R30" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S30" s="68" t="s">
         <v>104</v>
@@ -33860,7 +33878,7 @@
         <v>17</v>
       </c>
       <c r="R31" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S31" s="68" t="s">
         <v>94</v>
@@ -33909,7 +33927,7 @@
         <v>17</v>
       </c>
       <c r="R32" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S32" s="68" t="s">
         <v>80</v>
@@ -33929,7 +33947,7 @@
         <v>17</v>
       </c>
       <c r="R33" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S33" s="68" t="s">
         <v>88</v>
@@ -33949,7 +33967,7 @@
         <v>17</v>
       </c>
       <c r="R34" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S34" s="68" t="s">
         <v>93</v>
@@ -33969,7 +33987,7 @@
         <v>17</v>
       </c>
       <c r="R35" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S35" s="68" t="s">
         <v>92</v>
@@ -33989,7 +34007,7 @@
         <v>17</v>
       </c>
       <c r="R36" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S36" s="68" t="s">
         <v>86</v>
@@ -34009,7 +34027,7 @@
         <v>17</v>
       </c>
       <c r="R37" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S37" s="68" t="s">
         <v>83</v>
@@ -34029,7 +34047,7 @@
         <v>17</v>
       </c>
       <c r="R38" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S38" s="68" t="s">
         <v>82</v>
@@ -34049,7 +34067,7 @@
         <v>17</v>
       </c>
       <c r="R39" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S39" s="68" t="s">
         <v>79</v>
@@ -34069,7 +34087,7 @@
         <v>17</v>
       </c>
       <c r="R40" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S40" s="68" t="s">
         <v>155</v>
@@ -34089,7 +34107,7 @@
         <v>17</v>
       </c>
       <c r="R41" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S41" s="68" t="s">
         <v>105</v>
@@ -34109,7 +34127,7 @@
         <v>17</v>
       </c>
       <c r="R42" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S42" s="68" t="s">
         <v>91</v>
@@ -34129,7 +34147,7 @@
         <v>17</v>
       </c>
       <c r="R43" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S43" s="68" t="s">
         <v>101</v>
@@ -34149,7 +34167,7 @@
         <v>17</v>
       </c>
       <c r="R44" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S44" s="68" t="s">
         <v>93</v>
@@ -34169,7 +34187,7 @@
         <v>17</v>
       </c>
       <c r="R45" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S45" s="68" t="s">
         <v>88</v>
@@ -34186,7 +34204,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="S46" s="69" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="V46" s="70" t="n">
         <f aca="false">SUMIFS(V7:V45,R7:R45,"BUY")-SUMIFS(V7:V45,R7:R45,"SELL")</f>
@@ -34243,22 +34261,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="32" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34266,16 +34284,16 @@
         <v>69</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C6" s="26" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F6" s="26" t="s">
         <v>74</v>
@@ -34293,37 +34311,37 @@
         <v>10</v>
       </c>
       <c r="K6" s="26" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L6" s="26" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="M6" s="26" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N6" s="26" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O6" s="26" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="Q6" s="26" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="R6" s="26" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="S6" s="26" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="T6" s="26" t="s">
         <v>73</v>
       </c>
       <c r="U6" s="26" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="V6" s="26" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34379,10 +34397,10 @@
       </c>
       <c r="O7" s="67"/>
       <c r="Q7" s="68" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="R7" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S7" s="68" t="s">
         <v>82</v>
@@ -34450,10 +34468,10 @@
       </c>
       <c r="O8" s="67"/>
       <c r="Q8" s="68" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="R8" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S8" s="68" t="s">
         <v>83</v>
@@ -34521,10 +34539,10 @@
       </c>
       <c r="O9" s="67"/>
       <c r="Q9" s="68" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="R9" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S9" s="68" t="s">
         <v>79</v>
@@ -34592,7 +34610,7 @@
       </c>
       <c r="O10" s="67"/>
       <c r="S10" s="69" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="V10" s="70" t="n">
         <f aca="false">SUMIFS(V7:V9,R7:R9,"BUY")-SUMIFS(V7:V9,R7:R9,"SELL")</f>
@@ -35104,22 +35122,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="32" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35127,16 +35145,16 @@
         <v>69</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C6" s="27" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F6" s="27" t="s">
         <v>74</v>
@@ -35154,37 +35172,37 @@
         <v>10</v>
       </c>
       <c r="K6" s="27" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L6" s="27" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="M6" s="27" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N6" s="27" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O6" s="27" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="Q6" s="27" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="R6" s="27" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="S6" s="27" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="T6" s="27" t="s">
         <v>73</v>
       </c>
       <c r="U6" s="27" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="V6" s="27" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35240,10 +35258,10 @@
       </c>
       <c r="O7" s="67"/>
       <c r="Q7" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R7" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S7" s="68" t="s">
         <v>79</v>
@@ -35311,10 +35329,10 @@
       </c>
       <c r="O8" s="67"/>
       <c r="Q8" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R8" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S8" s="68" t="s">
         <v>82</v>
@@ -35382,10 +35400,10 @@
       </c>
       <c r="O9" s="67"/>
       <c r="Q9" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R9" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S9" s="68" t="s">
         <v>83</v>
@@ -35453,10 +35471,10 @@
       </c>
       <c r="O10" s="67"/>
       <c r="Q10" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R10" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S10" s="68" t="s">
         <v>80</v>
@@ -35523,13 +35541,13 @@
         <v>-12852</v>
       </c>
       <c r="O11" s="67" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="Q11" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R11" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S11" s="68" t="s">
         <v>86</v>
@@ -35596,13 +35614,13 @@
         <v>-8600</v>
       </c>
       <c r="O12" s="67" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="Q12" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R12" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S12" s="68" t="s">
         <v>93</v>
@@ -35670,10 +35688,10 @@
       </c>
       <c r="O13" s="67"/>
       <c r="Q13" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R13" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S13" s="68" t="s">
         <v>92</v>
@@ -35740,13 +35758,13 @@
         <v>8773</v>
       </c>
       <c r="O14" s="67" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q14" s="68" t="s">
+        <v>268</v>
+      </c>
+      <c r="R14" s="68" t="s">
         <v>203</v>
-      </c>
-      <c r="Q14" s="68" t="s">
-        <v>263</v>
-      </c>
-      <c r="R14" s="68" t="s">
-        <v>202</v>
       </c>
       <c r="S14" s="68" t="s">
         <v>96</v>
@@ -35814,10 +35832,10 @@
       </c>
       <c r="O15" s="67"/>
       <c r="Q15" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R15" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S15" s="68" t="s">
         <v>102</v>
@@ -35885,10 +35903,10 @@
       </c>
       <c r="O16" s="67"/>
       <c r="Q16" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R16" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S16" s="68" t="s">
         <v>94</v>
@@ -35956,10 +35974,10 @@
       </c>
       <c r="O17" s="67"/>
       <c r="Q17" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R17" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S17" s="68" t="s">
         <v>100</v>
@@ -36027,10 +36045,10 @@
       </c>
       <c r="O18" s="67"/>
       <c r="Q18" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R18" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S18" s="68" t="s">
         <v>104</v>
@@ -36098,10 +36116,10 @@
       </c>
       <c r="O19" s="67"/>
       <c r="Q19" s="68" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="R19" s="68" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S19" s="68" t="s">
         <v>88</v>
@@ -36169,7 +36187,7 @@
       </c>
       <c r="O20" s="67"/>
       <c r="S20" s="69" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="V20" s="70" t="n">
         <f aca="false">SUMIFS(V7:V19,R7:R19,"BUY")-SUMIFS(V7:V19,R7:R19,"SELL")</f>
@@ -36281,7 +36299,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="67" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36336,7 +36354,7 @@
         <v>448.5</v>
       </c>
       <c r="O23" s="67" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36497,7 +36515,7 @@
         <v>-422.2</v>
       </c>
       <c r="O26" s="67" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36628,17 +36646,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36646,16 +36664,16 @@
         <v>69</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C6" s="28" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F6" s="28" t="s">
         <v>74</v>
@@ -36673,19 +36691,19 @@
         <v>10</v>
       </c>
       <c r="K6" s="28" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L6" s="28" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="M6" s="28" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N6" s="28" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O6" s="28" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36696,7 +36714,7 @@
         <v>79</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D7" s="66" t="n">
         <v>915</v>
@@ -36749,7 +36767,7 @@
         <v>82</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D8" s="66" t="n">
         <v>792</v>
@@ -36802,7 +36820,7 @@
         <v>80</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D9" s="66" t="n">
         <v>59</v>
@@ -36855,7 +36873,7 @@
         <v>83</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D10" s="66" t="n">
         <v>337</v>
@@ -36908,7 +36926,7 @@
         <v>89</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D11" s="66" t="n">
         <v>800</v>
@@ -36952,7 +36970,7 @@
         <v>-24600</v>
       </c>
       <c r="O11" s="67" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37016,7 +37034,7 @@
         <v>84</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D13" s="66" t="n">
         <v>120</v>
@@ -37060,7 +37078,7 @@
         <v>-20226</v>
       </c>
       <c r="O13" s="67" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37071,7 +37089,7 @@
         <v>86</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D14" s="66" t="n">
         <v>1732</v>
@@ -37177,7 +37195,7 @@
         <v>93</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D16" s="66" t="n">
         <v>18</v>
@@ -37230,7 +37248,7 @@
         <v>88</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D17" s="66" t="n">
         <v>24</v>
@@ -37336,7 +37354,7 @@
         <v>92</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D19" s="66" t="n">
         <v>20</v>
@@ -37389,7 +37407,7 @@
         <v>106</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D20" s="66" t="n">
         <v>52</v>
@@ -37442,7 +37460,7 @@
         <v>94</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D21" s="66" t="n">
         <v>45</v>
@@ -37495,7 +37513,7 @@
         <v>96</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D22" s="66" t="n">
         <v>8</v>
@@ -37548,7 +37566,7 @@
         <v>100</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D23" s="66" t="n">
         <v>18</v>
@@ -37654,7 +37672,7 @@
         <v>114</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D25" s="66" t="n">
         <v>33</v>
@@ -37707,7 +37725,7 @@
         <v>117</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D26" s="66" t="n">
         <v>111</v>
@@ -37760,7 +37778,7 @@
         <v>102</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D27" s="66" t="n">
         <v>13</v>
@@ -37919,7 +37937,7 @@
         <v>85</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D30" s="66" t="n">
         <v>13</v>
@@ -38025,7 +38043,7 @@
         <v>123</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D32" s="66" t="n">
         <v>187</v>
@@ -38078,7 +38096,7 @@
         <v>124</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D33" s="66" t="n">
         <v>1072</v>
@@ -38131,7 +38149,7 @@
         <v>126</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D34" s="66" t="n">
         <v>19</v>
@@ -38184,7 +38202,7 @@
         <v>127</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D35" s="66" t="n">
         <v>110</v>
@@ -38228,7 +38246,7 @@
         <v>-2625.7</v>
       </c>
       <c r="O35" s="67" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -38239,7 +38257,7 @@
         <v>128</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D36" s="66" t="n">
         <v>302</v>
@@ -38292,7 +38310,7 @@
         <v>129</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D37" s="66" t="n">
         <v>166</v>
@@ -38345,7 +38363,7 @@
         <v>130</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D38" s="66" t="n">
         <v>116</v>
@@ -38398,7 +38416,7 @@
         <v>131</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D39" s="66" t="n">
         <v>33</v>
@@ -38451,7 +38469,7 @@
         <v>87</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D40" s="66" t="n">
         <v>5</v>
@@ -38495,7 +38513,7 @@
         <v>-5</v>
       </c>
       <c r="O40" s="67" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -38506,7 +38524,7 @@
         <v>132</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D41" s="66" t="n">
         <v>380</v>
@@ -38559,7 +38577,7 @@
         <v>133</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D42" s="66" t="n">
         <v>245</v>
@@ -38612,7 +38630,7 @@
         <v>134</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D43" s="66" t="n">
         <v>35</v>
@@ -38665,7 +38683,7 @@
         <v>136</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D44" s="66" t="n">
         <v>51</v>
@@ -38771,7 +38789,7 @@
         <v>137</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D46" s="66" t="n">
         <v>124</v>
@@ -38824,7 +38842,7 @@
         <v>138</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D47" s="66" t="n">
         <v>49</v>
@@ -38877,7 +38895,7 @@
         <v>141</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D48" s="66" t="n">
         <v>54</v>
@@ -38983,7 +39001,7 @@
         <v>143</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D50" s="66" t="n">
         <v>67</v>
@@ -39036,7 +39054,7 @@
         <v>139</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D51" s="66" t="n">
         <v>150</v>
@@ -39089,7 +39107,7 @@
         <v>145</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D52" s="66" t="n">
         <v>48</v>
@@ -39142,7 +39160,7 @@
         <v>147</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D53" s="66" t="n">
         <v>132</v>
@@ -39195,7 +39213,7 @@
         <v>149</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D54" s="66" t="n">
         <v>33</v>
@@ -39301,7 +39319,7 @@
         <v>153</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D56" s="66" t="n">
         <v>9</v>
@@ -39407,7 +39425,7 @@
         <v>161</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D58" s="66" t="n">
         <v>20</v>
@@ -39504,7 +39522,7 @@
         <v>0</v>
       </c>
       <c r="O59" s="67" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>